<commit_message>
Rebuild as AI-generated training plan hub; remove organisation references
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WjjLYmDSzttqv8ksfDSavR
</commit_message>
<xml_diff>
--- a/practice/CX_Complaints_Sample.xlsx
+++ b/practice/CX_Complaints_Sample.xlsx
@@ -508,7 +508,6 @@
           <t>New connection</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>Open</t>
@@ -626,7 +625,6 @@
           <t>Reconnection</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Open</t>
@@ -684,7 +682,6 @@
           <t>Reconnection</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Open</t>
@@ -862,7 +859,6 @@
           <t>Meter reading</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>Open</t>
@@ -950,7 +946,6 @@
           <t>Staff conduct</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1038,7 +1033,6 @@
           <t>Billing</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1126,7 +1120,6 @@
           <t>Meter reading</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1304,7 +1297,6 @@
           <t>Billing</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1632,7 +1624,6 @@
           <t>Billing</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1870,7 +1861,6 @@
           <t>New connection</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2078,7 +2068,6 @@
           <t>New connection</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2106,7 +2095,6 @@
           <t>Billing</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2344,7 +2332,6 @@
           <t>New connection</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2402,7 +2389,6 @@
           <t>Billing</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2460,7 +2446,6 @@
           <t>Billing</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2518,7 +2503,6 @@
           <t>Outage</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2576,7 +2560,6 @@
           <t>Billing</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2664,7 +2647,6 @@
           <t>Billing</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2692,7 +2674,6 @@
           <t>Reconnection</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2840,7 +2821,6 @@
           <t>Outage</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>Open</t>
@@ -2870,10 +2850,11 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Practice file for the JPS AI Productivity Workshop</t>
-        </is>
-      </c>
-    </row>
+          <t>Practice file for the AI Productivity Workshop</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -2884,7 +2865,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>All names, codes and figures are fictional. Do not replace them with real JPS data.</t>
+          <t>All names, codes and figures are fictional. Do not replace them with real company data.</t>
         </is>
       </c>
     </row>

</xml_diff>